<commit_message>
init step 4 - wan
</commit_message>
<xml_diff>
--- a/RFIDP2P3_Web/wwwroot/templates/Master Suffix to Unique.xlsx
+++ b/RFIDP2P3_Web/wwwroot/templates/Master Suffix to Unique.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\webproject\.Net\RFID-Frontend\RFIDP2P3_Web\wwwroot\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\webproject\RFID-Anbunka-Frontend\RFIDP2P3_Web\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B004DEAA-2277-4775-8198-A3D73E3F72F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F882D246-5FF9-4709-807D-E8B6BEBBDA9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="12196" xr2:uid="{976698CF-AFD0-4B0D-B1E3-268D4C624749}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Suffix</t>
   </si>
@@ -46,6 +46,12 @@
   </si>
   <si>
     <t>Xenia Export</t>
+  </si>
+  <si>
+    <t>Order From</t>
+  </si>
+  <si>
+    <t>KAP</t>
   </si>
 </sst>
 </file>
@@ -417,14 +423,14 @@
   <sheetPr codeName="Sheet1">
     <tabColor theme="0"/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15.265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -437,8 +443,11 @@
       <c r="D1" t="s">
         <v>0</v>
       </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -450,6 +459,9 @@
       </c>
       <c r="D2" t="s">
         <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add menu: order tmmin, order ddmi update: status master suffix, parameter capacity, process, result, summary capacity
</commit_message>
<xml_diff>
--- a/RFIDP2P3_Web/wwwroot/templates/Master Suffix to Unique.xlsx
+++ b/RFIDP2P3_Web/wwwroot/templates/Master Suffix to Unique.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\webproject\RFID-Anbunka-Frontend\RFIDP2P3_Web\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F882D246-5FF9-4709-807D-E8B6BEBBDA9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6544DA6-078B-422C-8F0B-FED0BB61491A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="12196" xr2:uid="{976698CF-AFD0-4B0D-B1E3-268D4C624749}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Suffix</t>
   </si>
@@ -52,6 +52,12 @@
   </si>
   <si>
     <t>KAP</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Active</t>
   </si>
 </sst>
 </file>
@@ -423,14 +429,15 @@
   <sheetPr codeName="Sheet1">
     <tabColor theme="0"/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15.265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.73046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -446,8 +453,11 @@
       <c r="E1" t="s">
         <v>7</v>
       </c>
+      <c r="F1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -462,6 +472,9 @@
       </c>
       <c r="E2" t="s">
         <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>